<commit_message>
added draft visuals and feedback from day 22
</commit_message>
<xml_diff>
--- a/data/global+EU-WHO-measles-by-year.xlsx
+++ b/data/global+EU-WHO-measles-by-year.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arkeshdas/Documents/CMSE 402/Semester Project/semester-project-arkeshdas/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F055E5FD-4285-6441-9710-273908C75386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22677D6D-A1C6-EF44-BB9A-FF4509AEAC88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="660" windowWidth="18200" windowHeight="8000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -468,12 +468,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -938,6 +939,9 @@
       <c r="B2" t="s">
         <v>3</v>
       </c>
+      <c r="C2" s="3">
+        <v>33998</v>
+      </c>
       <c r="D2" t="s">
         <v>4</v>
       </c>
@@ -1080,6 +1084,9 @@
       </c>
       <c r="B3" t="s">
         <v>3</v>
+      </c>
+      <c r="C3" s="3">
+        <v>425000</v>
       </c>
       <c r="D3" t="s">
         <v>50</v>

</xml_diff>